<commit_message>
v0.1.2: restore backup, add global rules, fix remote cmd frame length
- Restore project from backup (remove TM dynamic changes)
- CLAUDE.md: add Avoid Hardcoding global rule
- remote_command_panel.py: data_len now uses Excel config values directly
- enums.yaml: update from telemetry config import
</commit_message>
<xml_diff>
--- a/项目文档/通讯协议/excel版遥测大表/遥测配置表.xlsx
+++ b/项目文档/通讯协议/excel版遥测大表/遥测配置表.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codex Workspace\01_Projects\项目文档\通讯协议\excel版遥测大表\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF73D0E-4984-4E9B-8E7C-BC46D0FDAE52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E57D0B7-4A2D-4F43-97B9-5AD5F196CBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="TM1 参数表" sheetId="1" r:id="rId1"/>
-    <sheet name="TM2 参数表" sheetId="2" r:id="rId2"/>
-    <sheet name="查询包 参数表" sheetId="3" r:id="rId3"/>
+    <sheet name="常规包1参数表" sheetId="1" r:id="rId1"/>
+    <sheet name="常规包2参数表" sheetId="2" r:id="rId2"/>
+    <sheet name="查询包1参数表" sheetId="3" r:id="rId3"/>
+    <sheet name="查询包2参数表" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1400" uniqueCount="531">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1414" uniqueCount="531">
   <si>
     <t>序号</t>
   </si>
@@ -11419,4 +11420,59 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEFBA2A6-6BDF-41AF-BB34-FDE1795B9803}">
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetData>
+    <row r="1" spans="1:14" ht="58">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>